<commit_message>
Refactor(usuarios): Reestructurar la gestión de usuarios y mejorar la organización del código.
Feat(auth): Añadir FIROLID a la consulta de usuario para la identificación de roles.
Style(css): Reemplazar los estilos de interruptor por estilos de cargador.
Refactor(diseño): Consolidar los archivos de diseño en parciales y la plantilla principal.
Feat(panel): Añadir DashboardController con el método de plantilla.
Refactor(rutas): Simplificar las rutas de usuario y añadir rutas de panel.
Refactor(modelos): Actualizar UserModel con mejor validación y métodos.
Style(js): Limpiar y mejorar la funcionalidad de los scripts de usuario.
</commit_message>
<xml_diff>
--- a/public/assets/plantillas/carga_masiva_usuario.xlsx
+++ b/public/assets/plantillas/carga_masiva_usuario.xlsx
@@ -1,26 +1,132 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scorp\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2425B06-6008-4296-BAD6-AE73829C5B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="CargaMasivaUsuarios" sheetId="1" r:id="rId1"/>
+    <sheet name="CatSucursales" sheetId="2" r:id="rId2"/>
+    <sheet name="CatRoles" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Apellido Paterno</t>
+  </si>
+  <si>
+    <t>Apellido Materno</t>
+  </si>
+  <si>
+    <t>Correo Electronico</t>
+  </si>
+  <si>
+    <t>Clave</t>
+  </si>
+  <si>
+    <t>Rol ID</t>
+  </si>
+  <si>
+    <t>Rol Id</t>
+  </si>
+  <si>
+    <t>Estatus</t>
+  </si>
+  <si>
+    <t>Correo Verificado</t>
+  </si>
+  <si>
+    <t>Sucursal Id</t>
+  </si>
+  <si>
+    <t>Rogelio</t>
+  </si>
+  <si>
+    <t>Espinosa</t>
+  </si>
+  <si>
+    <t>Reyes</t>
+  </si>
+  <si>
+    <t>respinosa@gmail.com</t>
+  </si>
+  <si>
+    <t>#R35p1n0s4#</t>
+  </si>
+  <si>
+    <t>Efrain</t>
+  </si>
+  <si>
+    <t>Esponoza</t>
+  </si>
+  <si>
+    <t>eespinosa@gmail.com</t>
+  </si>
+  <si>
+    <t>#335p1n0s4#</t>
+  </si>
+  <si>
+    <t>Administardor</t>
+  </si>
+  <si>
+    <t>Gerente</t>
+  </si>
+  <si>
+    <t>Cajero</t>
+  </si>
+  <si>
+    <t>Vendedor</t>
+  </si>
+  <si>
+    <t>Almacenista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koomersys - Congreso </t>
+  </si>
+  <si>
+    <t>Koomersys - Congreso II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koomersys - Guadiana </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koomersys - San Francisco </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koomersys - La Ventanita </t>
+  </si>
+  <si>
+    <t>Sucursal ID</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +134,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,13 +174,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +470,235 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3">
+        <v>1</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="3">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{221C1926-A640-4D12-BDF2-653F4BF06F58}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{1DFB9C3D-3C2F-471B-B45F-3D8A47983147}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5E021E-CCE5-43F6-A2B0-C15C06B0A997}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>38000</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>38001</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>38002</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>38003</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>38004</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34CB9871-01C0-42AC-936B-B63FAC582E62}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>